<commit_message>
Cambio en query de precios
</commit_message>
<xml_diff>
--- a/Pricing/Inflacion USA.xlsx
+++ b/Pricing/Inflacion USA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcos.larran\Desktop\Github\Proyectos_Streamlit\Pricing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0707BB01-1208-411B-9537-A94B4765D902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9418A9D-1ED9-4192-A0E3-D903E76EB16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
Cambios en control de proveedores
</commit_message>
<xml_diff>
--- a/Pricing/Inflacion USA.xlsx
+++ b/Pricing/Inflacion USA.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcos.larran\Desktop\Github\Proyectos_Streamlit\Pricing\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9418A9D-1ED9-4192-A0E3-D903E76EB16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Mes</t>
   </si>
@@ -110,13 +104,16 @@
   </si>
   <si>
     <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,21 +176,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -231,7 +220,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -265,7 +254,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -300,10 +288,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -476,11 +463,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -488,7 +475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -496,7 +483,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -504,7 +491,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -512,7 +499,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -520,7 +507,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -528,7 +515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -536,7 +523,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -544,7 +531,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -552,7 +539,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -560,7 +547,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -568,7 +555,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -576,7 +563,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -584,7 +571,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -592,7 +579,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -600,7 +587,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -608,7 +595,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -616,7 +603,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -624,7 +611,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -632,7 +619,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -640,7 +627,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -648,7 +635,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -656,7 +643,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -664,7 +651,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -672,7 +659,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -680,7 +667,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -688,7 +675,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -696,7 +683,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -704,12 +691,20 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2">
       <c r="A29" t="s">
         <v>29</v>
       </c>
       <c r="B29">
         <v>0.6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Control para evitar error
</commit_message>
<xml_diff>
--- a/Pricing/Inflacion USA.xlsx
+++ b/Pricing/Inflacion USA.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Mes</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
   </si>
 </sst>
 </file>
@@ -464,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -707,6 +710,14 @@
         <v>0.5</v>
       </c>
     </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31">
+        <v>-0.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>